<commit_message>
Add 3D clustering function and update dictionary files for enhanced data processing
</commit_message>
<xml_diff>
--- a/Atlas/Dog/Czeibert_dictionary.xlsx
+++ b/Atlas/Dog/Czeibert_dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Faces_Hu\CommonFiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\dog_brain_toolkit\Atlas\Dog\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE36663B-7D6E-4C85-AE7B-D8F4010F3D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E9CE031-3A3A-4F3E-A446-2E0D42BB0B28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="labelsDogs" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -317,9 +316,6 @@
     <t>Latin</t>
   </si>
   <si>
-    <t>Abreviation</t>
-  </si>
-  <si>
     <t xml:space="preserve">gyrus frontalis L </t>
   </si>
   <si>
@@ -1014,6 +1010,9 @@
   </si>
   <si>
     <t>File2</t>
+  </si>
+  <si>
+    <t>Abbreviation</t>
   </si>
 </sst>
 </file>
@@ -1856,14 +1855,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F119"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="37.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="37.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1874,16 +1873,16 @@
         <v>93</v>
       </c>
       <c r="D1" t="s">
-        <v>94</v>
+        <v>326</v>
       </c>
       <c r="E1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F1" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1894,10 +1893,10 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1905,20 +1904,20 @@
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D3" t="s">
         <v>3</v>
       </c>
       <c r="E3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F3" t="str">
         <f>LEFT(E3, SEARCH(".nii.gz", E3) - 1)</f>
         <v>L_gFrontalis</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1926,20 +1925,20 @@
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D4" t="s">
         <v>4</v>
       </c>
       <c r="E4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F4" t="str">
         <f t="shared" ref="F4:F67" si="0">LEFT(E4, SEARCH(".nii.gz", E4) - 1)</f>
         <v>R_gFrontalis</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1947,20 +1946,20 @@
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D5" t="s">
         <v>5</v>
       </c>
       <c r="E5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F5" t="str">
         <f t="shared" si="0"/>
         <v>L_gProreus</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1968,20 +1967,20 @@
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D6" t="s">
         <v>6</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F6" t="str">
         <f t="shared" si="0"/>
         <v>R_gProreus</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1989,20 +1988,20 @@
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F7" t="str">
         <f t="shared" si="0"/>
         <v>L_gCompositusRostralis</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2010,20 +2009,20 @@
         <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D8" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F8" t="str">
         <f t="shared" si="0"/>
         <v>R_gCompositusRostralis</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2031,20 +2030,20 @@
         <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D9" t="s">
         <v>9</v>
       </c>
       <c r="E9" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F9" t="str">
         <f t="shared" si="0"/>
         <v>L_gPrecruciatus</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2052,20 +2051,20 @@
         <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D10" t="s">
         <v>10</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F10" t="str">
         <f t="shared" si="0"/>
         <v>R_gPrecruciatus</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2073,20 +2072,20 @@
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D11" t="s">
         <v>11</v>
       </c>
       <c r="E11" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F11" t="str">
         <f t="shared" si="0"/>
         <v>L_gPostcruciatus</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2094,20 +2093,20 @@
         <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F12" t="str">
         <f t="shared" si="0"/>
         <v>R_gPostcruciatus</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2115,20 +2114,20 @@
         <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D13" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F13" t="str">
         <f t="shared" si="0"/>
         <v>L_gMarginalis</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2136,20 +2135,20 @@
         <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F14" t="str">
         <f t="shared" si="0"/>
         <v>R_gMarginalis</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2157,20 +2156,20 @@
         <v>15</v>
       </c>
       <c r="C15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D15" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E15" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F15" t="str">
         <f t="shared" si="0"/>
         <v>L_gEctomarginalis</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2178,20 +2177,20 @@
         <v>16</v>
       </c>
       <c r="C16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D16" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F16" t="str">
         <f t="shared" si="0"/>
         <v>R_gEctomarginalis</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2199,20 +2198,20 @@
         <v>17</v>
       </c>
       <c r="C17" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D17" t="s">
         <v>17</v>
       </c>
       <c r="E17" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F17" t="str">
         <f t="shared" si="0"/>
         <v>L_gOccipitalis</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2220,20 +2219,20 @@
         <v>18</v>
       </c>
       <c r="C18" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D18" t="s">
         <v>18</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F18" t="str">
         <f t="shared" si="0"/>
         <v>R_gOccipitalis</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2241,20 +2240,20 @@
         <v>19</v>
       </c>
       <c r="C19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D19" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E19" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F19" t="str">
         <f t="shared" si="0"/>
         <v>L_gSuprasylviusRostralis</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2262,20 +2261,20 @@
         <v>20</v>
       </c>
       <c r="C20" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F20" t="str">
         <f t="shared" si="0"/>
         <v>R_gSuprasylviusRostralis</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2283,20 +2282,20 @@
         <v>21</v>
       </c>
       <c r="C21" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D21" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E21" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F21" t="str">
         <f t="shared" si="0"/>
         <v>L_gSuprasylviusMedius</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2304,20 +2303,20 @@
         <v>22</v>
       </c>
       <c r="C22" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D22" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F22" t="str">
         <f t="shared" si="0"/>
         <v>R_gSuprasylviusMedius</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2325,20 +2324,20 @@
         <v>23</v>
       </c>
       <c r="C23" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D23" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E23" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F23" t="str">
         <f t="shared" si="0"/>
         <v>L_gSuprasylviusCaudalis</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2346,20 +2345,20 @@
         <v>24</v>
       </c>
       <c r="C24" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D24" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F24" t="str">
         <f t="shared" si="0"/>
         <v>R_gSuprasylviusCaudalis</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2367,20 +2366,20 @@
         <v>25</v>
       </c>
       <c r="C25" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D25" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E25" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F25" t="str">
         <f t="shared" si="0"/>
         <v>L_gEctosylviusRostralis</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2388,20 +2387,20 @@
         <v>26</v>
       </c>
       <c r="C26" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D26" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F26" t="str">
         <f t="shared" si="0"/>
         <v>R_gEctosylviusRostralis</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2409,20 +2408,20 @@
         <v>27</v>
       </c>
       <c r="C27" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D27" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E27" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F27" t="str">
         <f t="shared" si="0"/>
         <v>L_gEctosylviusMedius</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2430,20 +2429,20 @@
         <v>28</v>
       </c>
       <c r="C28" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D28" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F28" t="str">
         <f t="shared" si="0"/>
         <v>R_gEctosylviusMedius</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2451,20 +2450,20 @@
         <v>29</v>
       </c>
       <c r="C29" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D29" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E29" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F29" t="str">
         <f t="shared" si="0"/>
         <v>L_gEctosylviusCaudalis</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2472,20 +2471,20 @@
         <v>30</v>
       </c>
       <c r="C30" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D30" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F30" t="str">
         <f t="shared" si="0"/>
         <v>R_gEctosylviusCaudalis</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2493,20 +2492,20 @@
         <v>31</v>
       </c>
       <c r="C31" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D31" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E31" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F31" t="str">
         <f t="shared" si="0"/>
         <v>L_gSylviusRostralis</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2514,20 +2513,20 @@
         <v>32</v>
       </c>
       <c r="C32" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D32" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F32" t="str">
         <f t="shared" si="0"/>
         <v>R_gSylviusRostralis</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2535,20 +2534,20 @@
         <v>33</v>
       </c>
       <c r="C33" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D33" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E33" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F33" t="str">
         <f t="shared" si="0"/>
         <v>L_gSylviusCaudalis</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2556,20 +2555,20 @@
         <v>34</v>
       </c>
       <c r="C34" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D34" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F34" t="str">
         <f t="shared" si="0"/>
         <v>R_gSylviusCaudalis</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2577,20 +2576,20 @@
         <v>35</v>
       </c>
       <c r="C35" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D35" t="s">
         <v>35</v>
       </c>
       <c r="E35" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F35" t="str">
         <f t="shared" si="0"/>
         <v>L_gCompositusCaudalis</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2598,20 +2597,20 @@
         <v>36</v>
       </c>
       <c r="C36" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D36" t="s">
         <v>36</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F36" t="str">
         <f t="shared" si="0"/>
         <v>R_gCompositusCaudalis</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2619,20 +2618,20 @@
         <v>37</v>
       </c>
       <c r="C37" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D37" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E37" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F37" t="str">
         <f t="shared" si="0"/>
         <v>L_gRectus</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2640,20 +2639,20 @@
         <v>38</v>
       </c>
       <c r="C38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D38" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F38" t="str">
         <f t="shared" si="0"/>
         <v>R_gRectus</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2661,20 +2660,20 @@
         <v>39</v>
       </c>
       <c r="C39" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D39" t="s">
         <v>39</v>
       </c>
       <c r="E39" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F39" t="str">
         <f t="shared" si="0"/>
         <v>L_gGenualis</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -2682,20 +2681,20 @@
         <v>40</v>
       </c>
       <c r="C40" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D40" t="s">
         <v>40</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F40" t="str">
         <f t="shared" si="0"/>
         <v>R_gGenualis</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2703,20 +2702,20 @@
         <v>41</v>
       </c>
       <c r="C41" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D41" t="s">
         <v>41</v>
       </c>
       <c r="E41" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F41" t="str">
         <f t="shared" si="0"/>
         <v>L_aSubcallosa</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2724,20 +2723,20 @@
         <v>42</v>
       </c>
       <c r="C42" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D42" t="s">
         <v>42</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F42" t="str">
         <f t="shared" si="0"/>
         <v>R_aSubcallosa</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2745,20 +2744,20 @@
         <v>43</v>
       </c>
       <c r="C43" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D43" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E43" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F43" t="str">
         <f t="shared" si="0"/>
         <v>L_gCinguli</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2766,20 +2765,20 @@
         <v>44</v>
       </c>
       <c r="C44" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D44" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F44" t="str">
         <f t="shared" si="0"/>
         <v>R_gCinguli</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2787,20 +2786,20 @@
         <v>45</v>
       </c>
       <c r="C45" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D45" t="s">
         <v>45</v>
       </c>
       <c r="E45" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F45" t="str">
         <f t="shared" si="0"/>
         <v>L_gPresplenialis</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2808,20 +2807,20 @@
         <v>46</v>
       </c>
       <c r="C46" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D46" t="s">
         <v>46</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="F46" t="str">
         <f t="shared" si="0"/>
         <v>R_gPresplenialis</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2829,20 +2828,20 @@
         <v>47</v>
       </c>
       <c r="C47" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D47" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E47" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F47" t="str">
         <f t="shared" si="0"/>
         <v>L_gSplenialis</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2850,20 +2849,20 @@
         <v>48</v>
       </c>
       <c r="C48" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D48" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F48" t="str">
         <f t="shared" si="0"/>
         <v>R_gSplenialis</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2871,20 +2870,20 @@
         <v>49</v>
       </c>
       <c r="C49" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D49" t="s">
         <v>49</v>
       </c>
       <c r="E49" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="F49" t="str">
         <f t="shared" si="0"/>
         <v>L_gParahippocampalis</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2892,20 +2891,20 @@
         <v>50</v>
       </c>
       <c r="C50" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D50" t="s">
         <v>50</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="F50" t="str">
         <f t="shared" si="0"/>
         <v>R_gParahippocampalis</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2913,20 +2912,20 @@
         <v>51</v>
       </c>
       <c r="C51" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D51" t="s">
         <v>51</v>
       </c>
       <c r="E51" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F51" t="str">
         <f t="shared" si="0"/>
         <v>L_hippocampus</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
@@ -2934,20 +2933,20 @@
         <v>52</v>
       </c>
       <c r="C52" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D52" t="s">
         <v>52</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="F52" t="str">
         <f t="shared" si="0"/>
         <v>R_hippocampus</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
@@ -2955,20 +2954,20 @@
         <v>53</v>
       </c>
       <c r="C53" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D53" t="s">
         <v>53</v>
       </c>
       <c r="E53" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F53" t="str">
         <f t="shared" si="0"/>
         <v>L_lPiriformis</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
@@ -2976,20 +2975,20 @@
         <v>54</v>
       </c>
       <c r="C54" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D54" t="s">
         <v>54</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F54" t="str">
         <f t="shared" si="0"/>
         <v>R_lPiriformis</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
@@ -2997,20 +2996,20 @@
         <v>55</v>
       </c>
       <c r="C55" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D55" t="s">
         <v>55</v>
       </c>
       <c r="E55" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="F55" t="str">
         <f t="shared" si="0"/>
         <v>L_tOlfactorium</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
@@ -3018,20 +3017,20 @@
         <v>56</v>
       </c>
       <c r="C56" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D56" t="s">
         <v>56</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="F56" t="str">
         <f t="shared" si="0"/>
         <v>R_tOlfactorium</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
@@ -3039,20 +3038,20 @@
         <v>57</v>
       </c>
       <c r="C57" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D57" t="s">
         <v>57</v>
       </c>
       <c r="E57" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F57" t="str">
         <f t="shared" si="0"/>
         <v>L_gDiagonalis</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
@@ -3060,20 +3059,20 @@
         <v>58</v>
       </c>
       <c r="C58" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D58" t="s">
         <v>58</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="F58" t="str">
         <f t="shared" si="0"/>
         <v>R_gDiagonalis</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
@@ -3081,20 +3080,20 @@
         <v>59</v>
       </c>
       <c r="C59" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D59" t="s">
         <v>59</v>
       </c>
       <c r="E59" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F59" t="str">
         <f t="shared" si="0"/>
         <v>L_gParaterminalis</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
@@ -3102,20 +3101,20 @@
         <v>60</v>
       </c>
       <c r="C60" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D60" t="s">
         <v>60</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F60" t="str">
         <f t="shared" si="0"/>
         <v>R_gParaterminalis</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
@@ -3123,20 +3122,20 @@
         <v>61</v>
       </c>
       <c r="C61" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D61" t="s">
         <v>61</v>
       </c>
       <c r="E61" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F61" t="str">
         <f t="shared" si="0"/>
         <v>L_gOlfactoriusLateralis</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
@@ -3144,20 +3143,20 @@
         <v>62</v>
       </c>
       <c r="C62" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D62" t="s">
         <v>62</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F62" t="str">
         <f t="shared" si="0"/>
         <v>R_gOlfactoriusLateralis</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
@@ -3165,20 +3164,20 @@
         <v>63</v>
       </c>
       <c r="C63" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D63" t="s">
         <v>63</v>
       </c>
       <c r="E63" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F63" t="str">
         <f t="shared" si="0"/>
         <v>L_Thalamus</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
@@ -3186,20 +3185,20 @@
         <v>64</v>
       </c>
       <c r="C64" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D64" t="s">
         <v>64</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="F64" t="str">
         <f t="shared" si="0"/>
         <v>R_Thalamus</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
@@ -3207,20 +3206,20 @@
         <v>65</v>
       </c>
       <c r="C65" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D65" t="s">
         <v>65</v>
       </c>
       <c r="E65" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="F65" t="str">
         <f t="shared" si="0"/>
         <v>L_bOlfactorius</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
@@ -3228,20 +3227,20 @@
         <v>66</v>
       </c>
       <c r="C66" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D66" t="s">
         <v>66</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F66" t="str">
         <f t="shared" si="0"/>
         <v>R_bOlfactorius</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
@@ -3249,20 +3248,20 @@
         <v>67</v>
       </c>
       <c r="C67" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D67" t="s">
         <v>67</v>
       </c>
       <c r="E67" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F67" t="str">
         <f t="shared" si="0"/>
         <v>L_nCaudatus</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
@@ -3270,20 +3269,20 @@
         <v>68</v>
       </c>
       <c r="C68" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D68" t="s">
         <v>68</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F68" t="str">
         <f t="shared" ref="F68:F119" si="1">LEFT(E68, SEARCH(".nii.gz", E68) - 1)</f>
         <v>R_nCaudatus</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
@@ -3291,20 +3290,20 @@
         <v>69</v>
       </c>
       <c r="C69" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D69" t="s">
         <v>69</v>
       </c>
       <c r="E69" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F69" t="str">
         <f t="shared" si="1"/>
         <v>L_InsularCortex</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
@@ -3312,20 +3311,20 @@
         <v>70</v>
       </c>
       <c r="C70" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D70" t="s">
         <v>70</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F70" t="str">
         <f t="shared" si="1"/>
         <v>R_InsularCortex</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
@@ -3339,14 +3338,14 @@
         <v>71</v>
       </c>
       <c r="E71" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="F71" t="str">
         <f t="shared" si="1"/>
         <v>b_Hypophysis</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
@@ -3354,20 +3353,20 @@
         <v>72</v>
       </c>
       <c r="C72" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D72" t="s">
         <v>72</v>
       </c>
       <c r="E72" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F72" t="str">
         <f t="shared" si="1"/>
         <v>b_VermisCerebelli</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
@@ -3381,14 +3380,14 @@
         <v>73</v>
       </c>
       <c r="E73" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="F73" t="str">
         <f t="shared" si="1"/>
         <v>b_Pons</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
@@ -3402,14 +3401,14 @@
         <v>74</v>
       </c>
       <c r="E74" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F74" t="str">
         <f t="shared" si="1"/>
         <v>b_MedullaOblongata</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
@@ -3417,20 +3416,20 @@
         <v>75</v>
       </c>
       <c r="C75" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D75" t="s">
         <v>75</v>
       </c>
       <c r="E75" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F75" t="str">
         <f t="shared" si="1"/>
         <v>b_MedullaSpinalis</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
@@ -3444,14 +3443,14 @@
         <v>76</v>
       </c>
       <c r="E76" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F76" t="str">
         <f t="shared" si="1"/>
         <v>b_Mesencephalon</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
@@ -3465,14 +3464,14 @@
         <v>77</v>
       </c>
       <c r="E77" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="F77" t="str">
         <f t="shared" si="1"/>
         <v>b_Diencephalon</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
@@ -3480,20 +3479,20 @@
         <v>78</v>
       </c>
       <c r="C78" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D78" t="s">
         <v>78</v>
       </c>
       <c r="E78" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F78" t="str">
         <f t="shared" si="1"/>
         <v>b_NervusOpticus</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
@@ -3501,20 +3500,20 @@
         <v>79</v>
       </c>
       <c r="C79" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D79" t="s">
         <v>79</v>
       </c>
       <c r="E79" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="F79" t="str">
         <f t="shared" si="1"/>
         <v>L_HemispheriumCerebelli</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
@@ -3522,20 +3521,20 @@
         <v>80</v>
       </c>
       <c r="C80" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D80" t="s">
         <v>80</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F80" t="str">
         <f t="shared" si="1"/>
         <v>R_HemispheriumCerebelli</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
@@ -3543,20 +3542,20 @@
         <v>81</v>
       </c>
       <c r="C81" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D81" t="s">
         <v>81</v>
       </c>
       <c r="E81" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F81" t="str">
         <f t="shared" si="1"/>
         <v>b_CommissuraRostralis</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>81</v>
       </c>
@@ -3564,20 +3563,20 @@
         <v>82</v>
       </c>
       <c r="C82" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D82" t="s">
         <v>82</v>
       </c>
       <c r="E82" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F82" t="str">
         <f t="shared" si="1"/>
         <v>L_PedunculusOlfactorius</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>82</v>
       </c>
@@ -3585,20 +3584,20 @@
         <v>83</v>
       </c>
       <c r="C83" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D83" t="s">
         <v>83</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F83" t="str">
         <f t="shared" si="1"/>
         <v>R_PedunculusOlfactorius</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>83</v>
       </c>
@@ -3606,20 +3605,20 @@
         <v>84</v>
       </c>
       <c r="C84" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D84" t="s">
         <v>84</v>
       </c>
       <c r="E84" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F84" t="str">
         <f t="shared" si="1"/>
         <v>L_aSeptalis</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>84</v>
       </c>
@@ -3627,20 +3626,20 @@
         <v>85</v>
       </c>
       <c r="C85" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D85" t="s">
         <v>85</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F85" t="str">
         <f t="shared" si="1"/>
         <v>R_aSeptalis</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>85</v>
       </c>
@@ -3648,20 +3647,20 @@
         <v>86</v>
       </c>
       <c r="C86" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D86" t="s">
         <v>86</v>
       </c>
       <c r="E86" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F86" t="str">
         <f t="shared" si="1"/>
         <v>L_nEtTractusSpinalisNerviTrigemini</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>86</v>
       </c>
@@ -3669,20 +3668,20 @@
         <v>87</v>
       </c>
       <c r="C87" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D87" t="s">
         <v>87</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F87" t="str">
         <f t="shared" si="1"/>
         <v>R_nEtTractusSpinalisNerviTrigemini</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>87</v>
       </c>
@@ -3690,20 +3689,20 @@
         <v>88</v>
       </c>
       <c r="C88" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D88" t="s">
         <v>88</v>
       </c>
       <c r="E88" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F88" t="str">
         <f t="shared" si="1"/>
         <v>L_nVentralisCaudalisThalamiParsMedialis</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>88</v>
       </c>
@@ -3711,20 +3710,20 @@
         <v>89</v>
       </c>
       <c r="C89" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D89" t="s">
         <v>89</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F89" t="str">
         <f t="shared" si="1"/>
         <v>R_nVentralisCaudalisThalamiParsMedialis</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>89</v>
       </c>
@@ -3732,20 +3731,20 @@
         <v>90</v>
       </c>
       <c r="C90" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D90" t="s">
         <v>90</v>
       </c>
       <c r="E90" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F90" t="str">
         <f t="shared" si="1"/>
         <v>L_Amygdala</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>90</v>
       </c>
@@ -3753,20 +3752,20 @@
         <v>91</v>
       </c>
       <c r="C91" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D91" t="s">
         <v>91</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F91" t="str">
         <f t="shared" si="1"/>
         <v>R_Amygdala</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
@@ -3780,250 +3779,250 @@
         <v>92</v>
       </c>
       <c r="E92" t="s">
+        <v>297</v>
+      </c>
+      <c r="F92" t="str">
+        <f t="shared" si="1"/>
+        <v>b_Encephalon</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E93" t="s">
         <v>298</v>
       </c>
-      <c r="F92" t="str">
-        <f t="shared" si="1"/>
-        <v>b_Encephalon</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E93" t="s">
+      <c r="F93" t="str">
+        <f t="shared" si="1"/>
+        <v>L_OccipitoTemporal</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E94" t="s">
         <v>299</v>
       </c>
-      <c r="F93" t="str">
-        <f t="shared" si="1"/>
-        <v>L_OccipitoTemporal</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E94" t="s">
+      <c r="F94" t="str">
+        <f t="shared" si="1"/>
+        <v>L_OccipitoTemporalGM</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E95" t="s">
         <v>300</v>
       </c>
-      <c r="F94" t="str">
-        <f t="shared" si="1"/>
-        <v>L_OccipitoTemporalGM</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E95" t="s">
+      <c r="F95" t="str">
+        <f t="shared" si="1"/>
+        <v>L_gEctosylvius</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="E96" t="s">
         <v>301</v>
       </c>
-      <c r="F95" t="str">
-        <f t="shared" si="1"/>
-        <v>L_gEctosylvius</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="E96" t="s">
+      <c r="F96" t="str">
+        <f t="shared" si="1"/>
+        <v>L_gPerisylvius</v>
+      </c>
+    </row>
+    <row r="97" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E97" t="s">
         <v>302</v>
       </c>
-      <c r="F96" t="str">
-        <f t="shared" si="1"/>
-        <v>L_gPerisylvius</v>
-      </c>
-    </row>
-    <row r="97" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E97" t="s">
+      <c r="F97" t="str">
+        <f t="shared" si="1"/>
+        <v>L_gSuprasylvius</v>
+      </c>
+    </row>
+    <row r="98" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E98" t="s">
         <v>303</v>
       </c>
-      <c r="F97" t="str">
-        <f t="shared" si="1"/>
-        <v>L_gSuprasylvius</v>
-      </c>
-    </row>
-    <row r="98" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E98" t="s">
+      <c r="F98" t="str">
+        <f t="shared" si="1"/>
+        <v>L_gSylvius</v>
+      </c>
+    </row>
+    <row r="99" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E99" t="s">
         <v>304</v>
       </c>
-      <c r="F98" t="str">
-        <f t="shared" si="1"/>
-        <v>L_gSylvius</v>
-      </c>
-    </row>
-    <row r="99" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E99" t="s">
+      <c r="F99" t="str">
+        <f t="shared" si="1"/>
+        <v>L_hypothalamus</v>
+      </c>
+    </row>
+    <row r="100" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E100" t="s">
         <v>305</v>
       </c>
-      <c r="F99" t="str">
-        <f t="shared" si="1"/>
-        <v>L_hypothalamus</v>
-      </c>
-    </row>
-    <row r="100" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E100" t="s">
+      <c r="F100" t="str">
+        <f t="shared" si="1"/>
+        <v>b_Amygdala</v>
+      </c>
+    </row>
+    <row r="101" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E101" t="s">
         <v>306</v>
       </c>
-      <c r="F100" t="str">
-        <f t="shared" si="1"/>
-        <v>b_Amygdala</v>
-      </c>
-    </row>
-    <row r="101" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E101" t="s">
+      <c r="F101" t="str">
+        <f t="shared" si="1"/>
+        <v>b_Cortex</v>
+      </c>
+    </row>
+    <row r="102" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E102" t="s">
         <v>307</v>
       </c>
-      <c r="F101" t="str">
-        <f t="shared" si="1"/>
-        <v>b_Cortex</v>
-      </c>
-    </row>
-    <row r="102" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E102" t="s">
+      <c r="F102" t="str">
+        <f t="shared" si="1"/>
+        <v>b_OccipitoTemporal</v>
+      </c>
+    </row>
+    <row r="103" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E103" t="s">
         <v>308</v>
       </c>
-      <c r="F102" t="str">
-        <f t="shared" si="1"/>
-        <v>b_OccipitoTemporal</v>
-      </c>
-    </row>
-    <row r="103" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E103" t="s">
+      <c r="F103" t="str">
+        <f t="shared" si="1"/>
+        <v>b_OccipitoTemporalGM</v>
+      </c>
+    </row>
+    <row r="104" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E104" t="s">
         <v>309</v>
       </c>
-      <c r="F103" t="str">
-        <f t="shared" si="1"/>
-        <v>b_OccipitoTemporalGM</v>
-      </c>
-    </row>
-    <row r="104" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E104" t="s">
+      <c r="F104" t="str">
+        <f t="shared" si="1"/>
+        <v>b_Subcortical</v>
+      </c>
+    </row>
+    <row r="105" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E105" t="s">
         <v>310</v>
       </c>
-      <c r="F104" t="str">
-        <f t="shared" si="1"/>
-        <v>b_Subcortical</v>
-      </c>
-    </row>
-    <row r="105" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E105" t="s">
+      <c r="F105" t="str">
+        <f t="shared" si="1"/>
+        <v>b_bOlfactorius</v>
+      </c>
+    </row>
+    <row r="106" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E106" t="s">
         <v>311</v>
       </c>
-      <c r="F105" t="str">
-        <f t="shared" si="1"/>
-        <v>b_bOlfactorius</v>
-      </c>
-    </row>
-    <row r="106" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E106" t="s">
+      <c r="F106" t="str">
+        <f t="shared" si="1"/>
+        <v>b_fullbrain</v>
+      </c>
+    </row>
+    <row r="107" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E107" t="s">
         <v>312</v>
       </c>
-      <c r="F106" t="str">
-        <f t="shared" si="1"/>
-        <v>b_fullbrain</v>
-      </c>
-    </row>
-    <row r="107" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E107" t="s">
+      <c r="F107" t="str">
+        <f t="shared" si="1"/>
+        <v>b_gCinguli</v>
+      </c>
+    </row>
+    <row r="108" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E108" t="s">
         <v>313</v>
       </c>
-      <c r="F107" t="str">
-        <f t="shared" si="1"/>
-        <v>b_gCinguli</v>
-      </c>
-    </row>
-    <row r="108" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E108" t="s">
+      <c r="F108" t="str">
+        <f t="shared" si="1"/>
+        <v>b_gEctosylvius</v>
+      </c>
+    </row>
+    <row r="109" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E109" t="s">
         <v>314</v>
       </c>
-      <c r="F108" t="str">
-        <f t="shared" si="1"/>
-        <v>b_gEctosylvius</v>
-      </c>
-    </row>
-    <row r="109" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E109" t="s">
+      <c r="F109" t="str">
+        <f t="shared" si="1"/>
+        <v>b_gEctosylviusCaudalis</v>
+      </c>
+    </row>
+    <row r="110" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E110" t="s">
         <v>315</v>
       </c>
-      <c r="F109" t="str">
-        <f t="shared" si="1"/>
-        <v>b_gEctosylviusCaudalis</v>
-      </c>
-    </row>
-    <row r="110" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E110" t="s">
+      <c r="F110" t="str">
+        <f t="shared" si="1"/>
+        <v>b_gEctosylviusMedius</v>
+      </c>
+    </row>
+    <row r="111" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E111" t="s">
         <v>316</v>
       </c>
-      <c r="F110" t="str">
-        <f t="shared" si="1"/>
-        <v>b_gEctosylviusMedius</v>
-      </c>
-    </row>
-    <row r="111" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E111" t="s">
+      <c r="F111" t="str">
+        <f t="shared" si="1"/>
+        <v>b_gPerisylvius</v>
+      </c>
+    </row>
+    <row r="112" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E112" t="s">
         <v>317</v>
       </c>
-      <c r="F111" t="str">
-        <f t="shared" si="1"/>
-        <v>b_gPerisylvius</v>
-      </c>
-    </row>
-    <row r="112" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E112" t="s">
+      <c r="F112" t="str">
+        <f t="shared" si="1"/>
+        <v>b_gPerisylvius2</v>
+      </c>
+    </row>
+    <row r="113" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E113" t="s">
         <v>318</v>
       </c>
-      <c r="F112" t="str">
-        <f t="shared" si="1"/>
-        <v>b_gPerisylvius2</v>
-      </c>
-    </row>
-    <row r="113" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E113" t="s">
+      <c r="F113" t="str">
+        <f t="shared" si="1"/>
+        <v>b_gSuprasylvius</v>
+      </c>
+    </row>
+    <row r="114" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E114" t="s">
         <v>319</v>
       </c>
-      <c r="F113" t="str">
-        <f t="shared" si="1"/>
-        <v>b_gSuprasylvius</v>
-      </c>
-    </row>
-    <row r="114" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E114" t="s">
+      <c r="F114" t="str">
+        <f t="shared" si="1"/>
+        <v>b_gSuprasylviusCaudalis</v>
+      </c>
+    </row>
+    <row r="115" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E115" t="s">
         <v>320</v>
       </c>
-      <c r="F114" t="str">
-        <f t="shared" si="1"/>
-        <v>b_gSuprasylviusCaudalis</v>
-      </c>
-    </row>
-    <row r="115" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E115" t="s">
+      <c r="F115" t="str">
+        <f t="shared" si="1"/>
+        <v>b_gSuprasylviusMedius</v>
+      </c>
+    </row>
+    <row r="116" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E116" t="s">
         <v>321</v>
       </c>
-      <c r="F115" t="str">
-        <f t="shared" si="1"/>
-        <v>b_gSuprasylviusMedius</v>
-      </c>
-    </row>
-    <row r="116" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E116" t="s">
+      <c r="F116" t="str">
+        <f t="shared" si="1"/>
+        <v>b_gSylvius</v>
+      </c>
+    </row>
+    <row r="117" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E117" t="s">
         <v>322</v>
       </c>
-      <c r="F116" t="str">
-        <f t="shared" si="1"/>
-        <v>b_gSylvius</v>
-      </c>
-    </row>
-    <row r="117" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E117" t="s">
+      <c r="F117" t="str">
+        <f t="shared" si="1"/>
+        <v>b_gSylviusCaudalis</v>
+      </c>
+    </row>
+    <row r="118" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E118" t="s">
         <v>323</v>
       </c>
-      <c r="F117" t="str">
-        <f t="shared" si="1"/>
-        <v>b_gSylviusCaudalis</v>
-      </c>
-    </row>
-    <row r="118" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E118" t="s">
+      <c r="F118" t="str">
+        <f t="shared" si="1"/>
+        <v>b_gSylviusRostralis</v>
+      </c>
+    </row>
+    <row r="119" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E119" t="s">
         <v>324</v>
-      </c>
-      <c r="F118" t="str">
-        <f t="shared" si="1"/>
-        <v>b_gSylviusRostralis</v>
-      </c>
-    </row>
-    <row r="119" spans="5:6" x14ac:dyDescent="0.3">
-      <c r="E119" t="s">
-        <v>325</v>
       </c>
       <c r="F119" t="str">
         <f t="shared" si="1"/>

</xml_diff>